<commit_message>
Fix CU ordering bugs, parallelize pipeline, add markdown audit
- Post-processing in export_to_excel.py:
  - _fix_header_order: rotate CU-misplaced grouped sub-columns
  - _fix_row_order: reinsert displaced children after parent headers
- Parallelized 5-PDF processing with ThreadPoolExecutor (~14 min vs ~50 min)
- Added markdown ground truth audit cell (107/110 checks pass, 97.3%)
- Known issues: GOOG BS empty lineItems, BNL combined Income+ComprehensiveIncome
- Analyzer schema: strengthened ordering descriptions for periodHeaders/rows
</commit_message>
<xml_diff>
--- a/output/excel/10K-MSFT-07-27-2023_classified.xlsx
+++ b/output/excel/10K-MSFT-07-27-2023_classified.xlsx
@@ -14,6 +14,11 @@
     <sheet name="05_BalanceSheet_balance_sheets" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="06_CashFlow_cash_flows_statemen" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="07_Equity_stockholders_equity_s" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="08_Equity_our_board_of_director" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="09_ComprehensiveIncome_the_foll" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="10_Equity_shares_of_common_stoc" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="11_Equity_we_repurchased_the_fo" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="12_Other_stock_based_compensati" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,7 +28,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -41,10 +46,6 @@
     </font>
     <font>
       <b val="1"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <sz val="10"/>
     </font>
   </fonts>
   <fills count="2">
@@ -77,7 +78,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -105,9 +106,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -474,7 +472,187 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:F6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="60" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Following are our monthly share repurchases for the fourth quarter of fiscal year 2023:  (in (In millions))</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Line Item</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Period</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Total Number of Shares Purchased</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Average Price Paid Per Share</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Total Number of Shares Purchased as Part of Publicly Announced Plans or Programs</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Approximate Dollar Value of Shares That May Yet Be Purchased Under the Plans or Programs</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   April 1, 2023 - April 30, 2023</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>April 1, 2023 - April 30, 2023</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>5,007,656</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>$ 287.97</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>5,007,656</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>$ 25,467</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   May 1, 2023 - May 31, 2023</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>May 1, 2023 - May 31, 2023</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>5,355,638</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>314.26</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>5,355,638</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>23,784</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   June 1, 2023 - June 30, 2023</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>June 1, 2023 - June 30, 2023</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>4,413,960</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>334.15</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>4,413,960</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>22,309</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   14,777,254</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>14,777,254</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>14,777,254</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr"/>
+      <c r="E6" s="7" t="inlineStr"/>
+      <c r="F6" s="7" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -486,7 +664,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Following are our monthly share repurchases for the fourth quarter of fiscal year 2023:  (in (In millions))</t>
+          <t>Shares of common stock outstanding were as follows:  (in (In millions))</t>
         </is>
       </c>
     </row>
@@ -498,123 +676,456 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>April 1, 2023 - April 30, 2023</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>May 1, 2023 - May 31, 2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>June 1, 2023 - June 30, 2023</t>
+          <t>2021</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Total Number of Shares Purchased</t>
+          <t xml:space="preserve">   Balance, beginning of year</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>5,007,656</t>
+          <t>7,464</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>5,355,638</t>
+          <t>7,519</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>4,413,960</t>
+          <t>7,571</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Average Price Paid Per Share</t>
+          <t xml:space="preserve">   Issued</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>$287.97</t>
+          <t>37</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>314.26</t>
+          <t>40</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>334.15</t>
+          <t>49</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>14,777,254</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>14,777,254</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="inlineStr"/>
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Repurchased</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>(69)</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>(95)</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>(101)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Balance, end of year</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>7,432</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>7,464</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>7,519</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="60" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>We repurchased the following shares of common stock under the share repurchase programs:  (in (In millions))</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Line Item</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Shares 2023</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Amount 2023</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Shares 2022</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Amount 2022</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Shares 2021</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>Amount 2021</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   First Quarter</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>$4,600</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>$6,200</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>$5,270</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Second Quarter</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>4,600</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>6,233</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>5,750</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Third Quarter</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>4,600</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>7,800</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>5,750</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Total Number of Shares Purchased as Part of Publicly Announced Plans or Programs</t>
+          <t xml:space="preserve">   Fourth Quarter</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>5,007,656</t>
+          <t>14</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>5,355,638</t>
+          <t>4,600</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>4,413,960</t>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>7,800</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>6,200</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>Approximate Dollar Value of Shares That May Yet Be Purchased Under the Plans or Programs</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>$25,467</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>23,784</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>22,309</t>
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Total</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>$18,400</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>95</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>$28,033</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>101</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>$22,970</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="60" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Stock-based compensation expense and related income tax benefits were as follows:  (in (In millions))</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Line Item</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Stock-based compensation expense</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>$9,611</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>$7,502</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>$6,118</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Income tax benefits related to stock-based compensation</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>1,651</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>1,293</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>1,065</t>
         </is>
       </c>
     </row>
@@ -685,7 +1196,7 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Dividends</t>
+          <t xml:space="preserve">   June 13, 2023</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
@@ -705,12 +1216,12 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>$0.68</t>
+          <t>$ 0.68</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>$5,054</t>
+          <t>$ 5,054</t>
         </is>
       </c>
     </row>
@@ -919,22 +1430,22 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>Gross margin</t>
-        </is>
-      </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Gross margin</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>146,052</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
+      <c r="C11" s="5" t="inlineStr">
         <is>
           <t>135,620</t>
         </is>
       </c>
-      <c r="D11" s="7" t="inlineStr">
+      <c r="D11" s="5" t="inlineStr">
         <is>
           <t>115,856</t>
         </is>
@@ -943,7 +1454,7 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Research and development</t>
+          <t xml:space="preserve">   Research and development</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
@@ -965,7 +1476,7 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Sales and marketing</t>
+          <t xml:space="preserve">   Sales and marketing</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
@@ -987,7 +1498,7 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>General and administrative</t>
+          <t xml:space="preserve">   General and administrative</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
@@ -1007,22 +1518,22 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>Operating income</t>
-        </is>
-      </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Operating income</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>88,523</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
         <is>
           <t>83,383</t>
         </is>
       </c>
-      <c r="D15" s="7" t="inlineStr">
+      <c r="D15" s="5" t="inlineStr">
         <is>
           <t>69,916</t>
         </is>
@@ -1031,7 +1542,7 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Other income, net</t>
+          <t xml:space="preserve">   Other income, net</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
@@ -1051,22 +1562,22 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t>Income before income taxes</t>
-        </is>
-      </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Income before income taxes</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>89,311</t>
         </is>
       </c>
-      <c r="C17" s="7" t="inlineStr">
+      <c r="C17" s="5" t="inlineStr">
         <is>
           <t>83,716</t>
         </is>
       </c>
-      <c r="D17" s="7" t="inlineStr">
+      <c r="D17" s="5" t="inlineStr">
         <is>
           <t>71,102</t>
         </is>
@@ -1075,7 +1586,7 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Provision for income taxes</t>
+          <t xml:space="preserve">   Provision for income taxes</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
@@ -1097,7 +1608,7 @@
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>Net income</t>
+          <t xml:space="preserve">   Net income</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
@@ -1238,7 +1749,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -1250,186 +1761,177 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>COMPREHENSIVE INCOME STATEMENTS
-(In millions)  (in In millions)</t>
+          <t>COMPREHENSIVE INCOME STATEMENTS  (in (In millions))</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="B2" s="10" t="inlineStr">
-        <is>
-          <t>Year Ended June 30,</t>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Line Item</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>2021</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Line Item</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>2023</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>2022</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>2021</t>
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Net income</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>$ 72,361</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>$ 72,738</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>$ 61,271</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>Net income</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>$ 72,361</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>$ 72,738</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>$ 61,271</t>
-        </is>
-      </c>
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>Other comprehensive income (loss), net of tax:</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr"/>
+      <c r="C4" s="9" t="inlineStr"/>
+      <c r="D4" s="9" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
-        <is>
-          <t>Other comprehensive income (loss), net of tax:</t>
-        </is>
-      </c>
-      <c r="B5" s="9" t="inlineStr"/>
-      <c r="C5" s="9" t="inlineStr"/>
-      <c r="D5" s="9" t="inlineStr"/>
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Net change related to derivatives</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>(14)</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Net change related to derivatives</t>
+          <t xml:space="preserve">   Net change related to investments</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>(14)</t>
+          <t>(1,444)</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>(5,360)</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>(2,266)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Net change related to investments</t>
+          <t xml:space="preserve">   Translation adjustments and other</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>(1,444)</t>
+          <t>(207)</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>(5,360)</t>
+          <t>(1,146)</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>(2,266)</t>
+          <t>873</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>Translation adjustments and other</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>(207)</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>(1,146)</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>873</t>
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Other comprehensive loss</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>(1,665)</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>(6,500)</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>(1,374)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>Other comprehensive loss</t>
+          <t>Comprehensive income</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>(1,665)</t>
+          <t>$ 70,696</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>(6,500)</t>
+          <t>$ 66,238</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>(1,374)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>Comprehensive income</t>
-        </is>
-      </c>
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>$ 70,696</t>
-        </is>
-      </c>
-      <c r="C10" s="7" t="inlineStr">
-        <is>
-          <t>$ 66,238</t>
-        </is>
-      </c>
-      <c r="D10" s="7" t="inlineStr">
-        <is>
           <t>$ 59,897</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="1">
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="B2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1464,12 +1966,12 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>June 30, 2023</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>June 30, 2022</t>
         </is>
       </c>
     </row>
@@ -1492,223 +1994,223 @@
       <c r="C4" s="9" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Total current assets</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>184,257</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>169,684</t>
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      Cash and cash equivalents</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>$ 34,704</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>$ 13,931</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Property and equipment, net of accumulated depreciation of $68,251 and $59,660</t>
+          <t xml:space="preserve">      Short-term investments</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>95,641</t>
+          <t>76,558</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>74,398</t>
+          <t>90,826</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Operating lease right-of-use assets</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>14,346</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>13,148</t>
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      Total cash, cash equivalents, and short-term investments</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>111,262</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>104,757</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Equity investments</t>
+          <t xml:space="preserve">      Accounts receivable, net of allowance for doubtful accounts of $650 and $633</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>9,879</t>
+          <t>48,688</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>6,891</t>
+          <t>44,261</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Goodwill</t>
+          <t xml:space="preserve">      Inventories</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>67,886</t>
+          <t>2,500</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>67,524</t>
+          <t>3,742</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Intangible assets, net</t>
+          <t xml:space="preserve">      Other current assets</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>9,366</t>
+          <t>21,807</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>11,298</t>
+          <t>16,924</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Other long-term assets</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>30,601</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>21,897</t>
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Total current assets</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>184,257</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>169,684</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">      Cash and cash equivalents</t>
+          <t xml:space="preserve">   Property and equipment, net of accumulated depreciation of $68,251 and $59,660</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>$34,704</t>
+          <t>95,641</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>$13,931</t>
+          <t>74,398</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">      Short-term investments</t>
+          <t xml:space="preserve">   Operating lease right-of-use assets</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>76,558</t>
+          <t>14,346</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>90,826</t>
+          <t>13,148</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      Total cash, cash equivalents, and short-term investments</t>
-        </is>
-      </c>
-      <c r="B14" s="7" t="inlineStr">
-        <is>
-          <t>111,262</t>
-        </is>
-      </c>
-      <c r="C14" s="7" t="inlineStr">
-        <is>
-          <t>104,757</t>
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Equity investments</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>9,879</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>6,891</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">      Accounts receivable, net of allowance for doubtful accounts of $650 and $633</t>
+          <t xml:space="preserve">   Goodwill</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>48,688</t>
+          <t>67,886</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>44,261</t>
+          <t>67,524</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">      Inventories</t>
+          <t xml:space="preserve">   Intangible assets, net</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>2,500</t>
+          <t>9,366</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>3,742</t>
+          <t>11,298</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">      Other current assets</t>
+          <t xml:space="preserve">   Other long-term assets</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>21,807</t>
+          <t>30,601</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>16,924</t>
+          <t>21,897</t>
         </is>
       </c>
     </row>
@@ -1720,12 +2222,12 @@
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>$411,976</t>
+          <t>$ 411,976</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>$364,840</t>
+          <t>$ 364,840</t>
         </is>
       </c>
     </row>
@@ -1748,223 +2250,223 @@
       <c r="C20" s="9" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Total current liabilities</t>
-        </is>
-      </c>
-      <c r="B21" s="7" t="inlineStr">
-        <is>
-          <t>104,149</t>
-        </is>
-      </c>
-      <c r="C21" s="7" t="inlineStr">
-        <is>
-          <t>95,082</t>
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      Accounts payable</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>$ 18,095</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>$ 19,000</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Long-term debt</t>
+          <t xml:space="preserve">      Current portion of long-term debt</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>41,990</t>
+          <t>5,247</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>47,032</t>
+          <t>2,749</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Long-term income taxes</t>
+          <t xml:space="preserve">      Accrued compensation</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>25,560</t>
+          <t>11,009</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>26,069</t>
+          <t>10,661</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Long-term unearned revenue</t>
+          <t xml:space="preserve">      Short-term income taxes</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>2,912</t>
+          <t>4,152</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>2,870</t>
+          <t>4,067</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Deferred income taxes</t>
+          <t xml:space="preserve">      Short-term unearned revenue</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>433</t>
+          <t>50,901</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>230</t>
+          <t>45,538</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Operating lease liabilities</t>
+          <t xml:space="preserve">      Other current liabilities</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>12,728</t>
+          <t>14,745</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>11,489</t>
+          <t>13,067</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Other long-term liabilities</t>
-        </is>
-      </c>
-      <c r="B27" s="5" t="inlineStr">
-        <is>
-          <t>17,981</t>
-        </is>
-      </c>
-      <c r="C27" s="5" t="inlineStr">
-        <is>
-          <t>15,526</t>
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Total current liabilities</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>104,149</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>95,082</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">      Accounts payable</t>
+          <t xml:space="preserve">   Long-term debt</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>$18,095</t>
+          <t>41,990</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>$19,000</t>
+          <t>47,032</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">      Current portion of long-term debt</t>
+          <t xml:space="preserve">   Long-term income taxes</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>5,247</t>
+          <t>25,560</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>2,749</t>
+          <t>26,069</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">      Accrued compensation</t>
+          <t xml:space="preserve">   Long-term unearned revenue</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>11,009</t>
+          <t>2,912</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>10,661</t>
+          <t>2,870</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">      Short-term income taxes</t>
+          <t xml:space="preserve">   Deferred income taxes</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>4,152</t>
+          <t>433</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>4,067</t>
+          <t>230</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">      Short-term unearned revenue</t>
+          <t xml:space="preserve">   Operating lease liabilities</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>50,901</t>
+          <t>12,728</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>45,538</t>
+          <t>11,489</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">      Other current liabilities</t>
+          <t xml:space="preserve">   Other long-term liabilities</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>14,745</t>
+          <t>17,981</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>13,067</t>
+          <t>15,526</t>
         </is>
       </c>
     </row>
@@ -1986,13 +2488,13 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="4" t="inlineStr">
+      <c r="A35" s="8" t="inlineStr">
         <is>
           <t>Commitments and contingencies</t>
         </is>
       </c>
-      <c r="B35" s="5" t="inlineStr"/>
-      <c r="C35" s="5" t="inlineStr"/>
+      <c r="B35" s="9" t="inlineStr"/>
+      <c r="C35" s="9" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="8" t="inlineStr">
@@ -2079,12 +2581,12 @@
       </c>
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>$411,976</t>
+          <t>$ 411,976</t>
         </is>
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>$364,840</t>
+          <t>$ 364,840</t>
         </is>
       </c>
     </row>
@@ -2183,320 +2685,320 @@
       <c r="D5" s="9" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Changes in operating assets and liabilities:</t>
-        </is>
-      </c>
-      <c r="B6" s="9" t="inlineStr"/>
-      <c r="C6" s="9" t="inlineStr"/>
-      <c r="D6" s="9" t="inlineStr"/>
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      Depreciation, amortization, and other</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>13,861</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>14,460</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>11,686</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Net cash from operations</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>87,582</t>
-        </is>
-      </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>89,035</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr">
-        <is>
-          <t>76,740</t>
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      Stock-based compensation expense</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>9,611</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>7,502</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>6,118</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">      Depreciation, amortization, and other</t>
+          <t xml:space="preserve">      Net recognized losses (gains) on investments and derivatives</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>13,861</t>
+          <t>196</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>14,460</t>
+          <t>(409)</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>11,686</t>
+          <t>(1,249)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">      Stock-based compensation expense</t>
+          <t xml:space="preserve">      Deferred income taxes</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>9,611</t>
+          <t>(6,059)</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>7,502</t>
+          <t>(5,702)</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>6,118</t>
+          <t>(150)</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      Net recognized losses (gains) on investments and derivatives</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>196</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>(409)</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>(1,249)</t>
-        </is>
-      </c>
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Changes in operating assets and liabilities:</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr"/>
+      <c r="C10" s="9" t="inlineStr"/>
+      <c r="D10" s="9" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">      Deferred income taxes</t>
+          <t xml:space="preserve">      Accounts receivable</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>(6,059)</t>
+          <t>(4,087)</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>(5,702)</t>
+          <t>(6,834)</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>(150)</t>
+          <t>(6,481)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">      Accounts receivable</t>
+          <t xml:space="preserve">      Inventories</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>(4,087)</t>
+          <t>1,242</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>(6,834)</t>
+          <t>(1,123)</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>(6,481)</t>
+          <t>(737)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">      Inventories</t>
+          <t xml:space="preserve">      Other current assets</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>1,242</t>
+          <t>(1,991)</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>(1,123)</t>
+          <t>(709)</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>(737)</t>
+          <t>(932)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">      Other current assets</t>
+          <t xml:space="preserve">      Other long-term assets</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>(1,991)</t>
+          <t>(2,833)</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>(709)</t>
+          <t>(2,805)</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>(932)</t>
+          <t>(3,459)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">      Other long-term assets</t>
+          <t xml:space="preserve">      Accounts payable</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>(2,833)</t>
+          <t>(2,721)</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>(2,805)</t>
+          <t>2,943</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>(3,459)</t>
+          <t>2,798</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">      Accounts payable</t>
+          <t xml:space="preserve">      Unearned revenue</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>(2,721)</t>
+          <t>5,535</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>2,943</t>
+          <t>5,109</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>2,798</t>
+          <t>4,633</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">      Unearned revenue</t>
+          <t xml:space="preserve">      Income taxes</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>5,535</t>
+          <t>(358)</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>5,109</t>
+          <t>696</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>4,633</t>
+          <t>(2,309)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">      Income taxes</t>
+          <t xml:space="preserve">      Other current liabilities</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>(358)</t>
+          <t>2,272</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>696</t>
+          <t>2,344</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>(2,309)</t>
+          <t>4,149</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">      Other current liabilities</t>
+          <t xml:space="preserve">      Other long-term liabilities</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>2,272</t>
+          <t>553</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>2,344</t>
+          <t>825</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>4,149</t>
+          <t>1,402</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      Other long-term liabilities</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>553</t>
-        </is>
-      </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>825</t>
-        </is>
-      </c>
-      <c r="D20" s="5" t="inlineStr">
-        <is>
-          <t>1,402</t>
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Net cash from operations</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>87,582</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>89,035</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>76,740</t>
         </is>
       </c>
     </row>
@@ -2895,22 +3397,22 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="6" t="inlineStr">
+      <c r="A40" s="4" t="inlineStr">
         <is>
           <t>Cash and cash equivalents, end of period</t>
         </is>
       </c>
-      <c r="B40" s="7" t="inlineStr">
+      <c r="B40" s="5" t="inlineStr">
         <is>
           <t>$ 34,704</t>
         </is>
       </c>
-      <c r="C40" s="7" t="inlineStr">
+      <c r="C40" s="5" t="inlineStr">
         <is>
           <t>$ 13,931</t>
         </is>
       </c>
-      <c r="D40" s="7" t="inlineStr">
+      <c r="D40" s="5" t="inlineStr">
         <is>
           <t>$ 14,224</t>
         </is>
@@ -2942,8 +3444,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>STOCKHOLDERS' EQUITY STATEMENTS
-(In millions, except per share amounts)  (in In millions, except per share amounts)</t>
+          <t>STOCKHOLDERS' EQUITY STATEMENTS  (in In millions, except per share amounts)</t>
         </is>
       </c>
     </row>
@@ -2980,27 +3481,24 @@
       <c r="D3" s="9" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">   Balance, beginning of period</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>$
-86,939</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>$
-83,111</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>$
-80,552</t>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>$ 86,939</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>$ 83,111</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>$ 80,552</t>
         </is>
       </c>
     </row>
@@ -3125,22 +3623,22 @@
       <c r="D10" s="9" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">   Balance, beginning of period</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>84,281</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C11" s="7" t="inlineStr">
         <is>
           <t>57,055</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="D11" s="7" t="inlineStr">
         <is>
           <t>34,566</t>
         </is>
@@ -3267,22 +3765,22 @@
       <c r="D17" s="9" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="4" t="inlineStr">
+      <c r="A18" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">   Balance, beginning of period</t>
         </is>
       </c>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B18" s="7" t="inlineStr">
         <is>
           <t>(4,678)</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
+      <c r="C18" s="7" t="inlineStr">
         <is>
           <t>1,822</t>
         </is>
       </c>
-      <c r="D18" s="5" t="inlineStr">
+      <c r="D18" s="7" t="inlineStr">
         <is>
           <t>3,186</t>
         </is>
@@ -3362,20 +3860,17 @@
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>$
-206,223</t>
+          <t>$ 206,223</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>$
-166,542</t>
+          <t>$ 166,542</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>$
-141,988</t>
+          <t>$ 141,988</t>
         </is>
       </c>
     </row>
@@ -3387,20 +3882,317 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>$
-2.72</t>
+          <t>$ 2.72</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>$
-2.48</t>
+          <t>$ 2.48</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>$
-2.24</t>
+          <t>$ 2.24</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="60" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Our Board of Directors declared the following dividends:</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Line Item</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Declaration Date</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Record Date</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Payment Date</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Dividend Per Share</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   September 20, 2022</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>September 20, 2022</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>November 17, 2022</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>December 8, 2022</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>$0.68</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>$5,066</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   November 29, 2022</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>November 29, 2022</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>February 16, 2023</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>March 9, 2023</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>0.68</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>5,059</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   March 14, 2023</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>March 14, 2023</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>May 18, 2023</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>June 8, 2023</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>0.68</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>5,054</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   June 13, 2023</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>June 13, 2023</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>August 17, 2023</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>September 14, 2023</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>0.68</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>5,054</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Total</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>$2.72</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>$20,233</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr"/>
+      <c r="F7" s="7" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="60" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>The following table summarizes the changes in accumulated other comprehensive income (loss) by component:  (in (In millions))</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Line Item</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Derivatives</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr"/>
+      <c r="C3" s="9" t="inlineStr"/>
+      <c r="D3" s="9" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Balance, beginning of period</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>$(13)</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>$(19)</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>$(38)</t>
         </is>
       </c>
     </row>

</xml_diff>